<commit_message>
test: update automation workflow and test assets
</commit_message>
<xml_diff>
--- a/tests/TestCase/EasyCMS_后台管理_接口测试用例.xlsx
+++ b/tests/TestCase/EasyCMS_后台管理_接口测试用例.xlsx
@@ -503,10 +503,8 @@
           <t>用例总数</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>97</t>
-        </is>
+      <c r="B4" s="2" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="5">
@@ -545,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L98"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4222,2520 +4220,2648 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>API-057A</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>角色管理</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/roles/{id}</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>口径</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>启用与停用用户统计字段按状态精确计数</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>目标角色已绑定启用、停用、锁定、未激活四类用户</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>1. 调用角色详情接口
+2. 分别核对 active_user_count 与 disabled_user_count
+3. 对照绑定用户状态分布</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>id=role_detail_stats_id</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>active_user_count 仅统计 status=1；disabled_user_count 仅统计 status=2；status=3/4 不计入这两个新增字段。</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>需求差异 DIFF_role_detail_user_status_counts §3/§6；接口文档 §14 角色详情</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>API-057B</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>角色管理</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>/api/v1/admin/roles/{id}</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>回归</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>新增状态统计字段后 user_count 原口径保持不变</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>目标角色已绑定多种状态用户</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>1. 调用角色详情接口
+2. 核对 user_count
+3. 与角色实际绑定用户总数比对</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>id=role_detail_stats_id</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>user_count 仍等于角色绑定用户总数，不因新增 active_user_count、disabled_user_count 而改变口径。</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>需求差异 DIFF_role_detail_user_status_counts §3/§6；接口文档 §14 角色详情</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>API-058</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>异常</t>
         </is>
       </c>
-      <c r="G59" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>不存在角色返回 1004</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
+      <c r="H61" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>1. 查询不存在角色 id
 2. 检查响应</t>
         </is>
       </c>
-      <c r="J59" s="2" t="inlineStr">
+      <c r="J61" s="2" t="inlineStr">
         <is>
           <t>id=999999</t>
         </is>
       </c>
-      <c r="K59" s="2" t="inlineStr">
+      <c r="K61" s="2" t="inlineStr">
         <is>
           <t>返回 1004。</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>接口文档-公共错误码；接口文档 §14 角色详情</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>API-059</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C60" s="2" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles</t>
         </is>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G60" s="2" t="inlineStr">
+      <c r="G62" s="2" t="inlineStr">
         <is>
           <t>新建角色成功</t>
         </is>
       </c>
-      <c r="H60" s="2" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
         <is>
           <t>具备 admin:roles:create 权限</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>1. 提交合法角色名称、编码、状态
 2. 检查返回</t>
         </is>
       </c>
-      <c r="J60" s="2" t="inlineStr">
+      <c r="J62" s="2" t="inlineStr">
         <is>
           <t>{"name":"内容审核员","code":"content_reviewer","description":"负责内容技术审核","status":1}</t>
         </is>
       </c>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="K62" s="2" t="inlineStr">
         <is>
           <t>返回“角色创建成功”；数据入库。</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="L62" s="2" t="inlineStr">
         <is>
           <t>接口文档 §15 新建角色；PRD §3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>API-060</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G61" s="2" t="inlineStr">
+      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>角色名称重复时阻止保存</t>
         </is>
       </c>
-      <c r="H61" s="2" t="inlineStr">
+      <c r="H63" s="2" t="inlineStr">
         <is>
           <t>已存在同名角色</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
+      <c r="I63" s="2" t="inlineStr">
         <is>
           <t>1. 使用重复 name 创建角色
 2. 检查响应</t>
         </is>
       </c>
-      <c r="J61" s="2" t="inlineStr">
+      <c r="J63" s="2" t="inlineStr">
         <is>
           <t>{"name":"系统管理员","code":"system_admin_copy","status":1}</t>
         </is>
       </c>
-      <c r="K61" s="2" t="inlineStr">
+      <c r="K63" s="2" t="inlineStr">
         <is>
           <t>返回 1001，message 为“角色名称已存在”。</t>
         </is>
       </c>
-      <c r="L61" s="2" t="inlineStr">
+      <c r="L63" s="2" t="inlineStr">
         <is>
           <t>接口文档 §15 新建角色；PRD §3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>API-061</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles</t>
         </is>
       </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="G64" s="2" t="inlineStr">
         <is>
           <t>角色编码重复时阻止保存</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr">
+      <c r="H64" s="2" t="inlineStr">
         <is>
           <t>已存在同编码角色</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>1. 使用重复 code 创建角色
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J62" s="2" t="inlineStr">
+      <c r="J64" s="2" t="inlineStr">
         <is>
           <t>{"name":"审核员副本","code":"system_admin","status":1}</t>
         </is>
       </c>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="K64" s="2" t="inlineStr">
         <is>
           <t>返回 1001，message 为“角色编码已存在”。</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr">
+      <c r="L64" s="2" t="inlineStr">
         <is>
           <t>接口文档 §15 新建角色；PRD §3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>API-062</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G63" s="2" t="inlineStr">
+      <c r="G65" s="2" t="inlineStr">
         <is>
           <t>角色编码格式非法时阻止保存</t>
         </is>
       </c>
-      <c r="H63" s="2" t="inlineStr">
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
+      <c r="I65" s="2" t="inlineStr">
         <is>
           <t>1. 提交包含大写或连字符的 code
 2. 检查响应</t>
         </is>
       </c>
-      <c r="J63" s="2" t="inlineStr">
+      <c r="J65" s="2" t="inlineStr">
         <is>
           <t>{"name":"审核员","code":"Content-Reviewer","status":1}</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr">
+      <c r="K65" s="2" t="inlineStr">
         <is>
           <t>返回 1001，提示编码仅允许小写字母、数字和下划线。</t>
         </is>
       </c>
-      <c r="L63" s="2" t="inlineStr">
+      <c r="L65" s="2" t="inlineStr">
         <is>
           <t>接口文档 §15 新建角色</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>API-063</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G64" s="2" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>编辑角色成功</t>
         </is>
       </c>
-      <c r="H64" s="2" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>存在目标角色</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>1. 修改角色名称、描述、状态
 2. 提交</t>
         </is>
       </c>
-      <c r="J64" s="2" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>{"name":"内容审核员-高级","description":"高级审核","status":1}</t>
         </is>
       </c>
-      <c r="K64" s="2" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>角色信息更新成功。</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>接口文档 §16 编辑角色</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>API-064</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G65" s="2" t="inlineStr">
+      <c r="G67" s="2" t="inlineStr">
         <is>
           <t>编辑角色时传 code 也应被忽略</t>
         </is>
       </c>
-      <c r="H65" s="2" t="inlineStr">
+      <c r="H67" s="2" t="inlineStr">
         <is>
           <t>存在目标角色</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
+      <c r="I67" s="2" t="inlineStr">
         <is>
           <t>1. 在编辑请求中附带 code
 2. 查询详情</t>
         </is>
       </c>
-      <c r="J65" s="2" t="inlineStr">
+      <c r="J67" s="2" t="inlineStr">
         <is>
           <t>{"name":"内容审核员","description":"说明","status":1,"code":"changed_code"}</t>
         </is>
       </c>
-      <c r="K65" s="2" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
         <is>
           <t>编码保持原值不变。</t>
         </is>
       </c>
-      <c r="L65" s="2" t="inlineStr">
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>接口文档 §16 编辑角色；接口差异提醒第 10 条</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>API-065</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/copy</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr">
         <is>
           <t>复制角色成功并继承原权限集</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H68" s="2" t="inlineStr">
         <is>
           <t>存在源角色且已配置权限</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="I68" s="2" t="inlineStr">
         <is>
           <t>1. 调用复制角色接口
 2. 查询新角色权限</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="J68" s="2" t="inlineStr">
         <is>
           <t>{"name":"内容审核员（副本）","code":"content_reviewer_copy"}</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr">
         <is>
           <t>返回创建成功；新角色拥有与源角色相同的权限配置。</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>接口文档 §17 复制角色；PRD §3.3.1/§3.5.2</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>API-066</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/copy</t>
         </is>
       </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G67" s="2" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr">
         <is>
           <t>复制角色时新名称或新编码重复被拦截</t>
         </is>
       </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="H69" s="2" t="inlineStr">
         <is>
           <t>存在源角色</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>1. 使用已存在的 name 或 code 复制角色
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J67" s="2" t="inlineStr">
+      <c r="J69" s="2" t="inlineStr">
         <is>
           <t>{"name":"系统管理员","code":"system_admin"}</t>
         </is>
       </c>
-      <c r="K67" s="2" t="inlineStr">
+      <c r="K69" s="2" t="inlineStr">
         <is>
           <t>返回 1001，指出重复字段。</t>
         </is>
       </c>
-      <c r="L67" s="2" t="inlineStr">
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>接口文档 §17 复制角色；接口文档 §15 错误响应</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>API-067</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C68" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/status</t>
         </is>
       </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G68" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>停用无活跃用户绑定的角色成功</t>
         </is>
       </c>
-      <c r="H68" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>目标角色无启用状态绑定用户</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>1. 提交 status=2
 2. 查询角色状态</t>
         </is>
       </c>
-      <c r="J68" s="2" t="inlineStr">
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>{"status":2}</t>
         </is>
       </c>
-      <c r="K68" s="2" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr">
         <is>
           <t>角色成功停用。</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>接口文档 §18 切换角色状态；PRD §3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>API-068</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/status</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr">
         <is>
           <t>停用存在活跃用户的角色时被拦截</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>目标角色已绑定启用中的用户</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>1. 提交 status=2
 2. 检查错误提示</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>{"status":2}</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr">
         <is>
           <t>返回 1005，message 说明存在 N 个活跃用户，需要先解绑或停用用户。</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>接口文档 §18 切换角色状态；PRD §3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>API-069</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G70" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>删除未绑定用户且非系统预置角色成功</t>
         </is>
       </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>目标角色满足删除条件</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>1. 调用删除接口
 2. 校验角色已不存在</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>id=deletable_role_id</t>
         </is>
       </c>
-      <c r="K70" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>返回“角色已删除”；data=null。</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>接口文档 §19 删除角色；PRD §3.3.2/§3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>API-070</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G71" s="2" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr">
         <is>
           <t>系统预置角色不可删除</t>
         </is>
       </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H73" s="2" t="inlineStr">
         <is>
           <t>目标角色 is_system_preset=true</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>1. 删除系统预置角色
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J71" s="2" t="inlineStr">
+      <c r="J73" s="2" t="inlineStr">
         <is>
           <t>id=1</t>
         </is>
       </c>
-      <c r="K71" s="2" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr">
         <is>
           <t>返回 1005，message 为“系统预置角色不可删除”。</t>
         </is>
       </c>
-      <c r="L71" s="2" t="inlineStr">
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>接口文档 §19 删除角色；PRD §3.3.1</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>API-071</t>
         </is>
       </c>
-      <c r="B72" s="2" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>角色管理</t>
         </is>
       </c>
-      <c r="C72" s="2" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}</t>
         </is>
       </c>
-      <c r="D72" s="2" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G72" s="2" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr">
         <is>
           <t>已绑定用户的角色不可删除</t>
         </is>
       </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H74" s="2" t="inlineStr">
         <is>
           <t>目标角色存在绑定用户</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>1. 删除已绑定用户的角色
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J72" s="2" t="inlineStr">
+      <c r="J74" s="2" t="inlineStr">
         <is>
           <t>id=bound_role_id</t>
         </is>
       </c>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
         <is>
           <t>返回 1005，message 表示需先解绑用户后再删除。</t>
         </is>
       </c>
-      <c r="L72" s="2" t="inlineStr">
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>接口文档 §19 删除角色；PRD §3.3.2/§3.3.3</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>API-072</t>
         </is>
       </c>
-      <c r="B73" s="2" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C73" s="2" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/permissions</t>
         </is>
       </c>
-      <c r="D73" s="2" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G73" s="2" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr">
         <is>
           <t>获取角色已绑定权限成功</t>
         </is>
       </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H75" s="2" t="inlineStr">
         <is>
           <t>存在目标角色</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>1. 调用角色权限查询接口
 2. 检查 permissions 列表</t>
         </is>
       </c>
-      <c r="J73" s="2" t="inlineStr">
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>id=1</t>
         </is>
       </c>
-      <c r="K73" s="2" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
         <is>
           <t>返回 role_id 与 permissions 数组；用于权限配置页回显。</t>
         </is>
       </c>
-      <c r="L73" s="2" t="inlineStr">
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>接口文档 §20 获取角色已绑定权限；PRD §3.5.2</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>API-073</t>
         </is>
       </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/permissions</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G74" s="2" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr">
         <is>
           <t>未配置任何权限的角色返回空数组</t>
         </is>
       </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H76" s="2" t="inlineStr">
         <is>
           <t>准备无权限角色</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>1. 调用角色权限查询接口
 2. 查看 permissions</t>
         </is>
       </c>
-      <c r="J74" s="2" t="inlineStr">
+      <c r="J76" s="2" t="inlineStr">
         <is>
           <t>id=no_permission_role_id</t>
         </is>
       </c>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr">
         <is>
           <t>permissions=[]，不返回 null。</t>
         </is>
       </c>
-      <c r="L74" s="2" t="inlineStr">
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>接口文档 §20 获取角色已绑定权限</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>API-074</t>
         </is>
       </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/permissions</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G75" s="2" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>更新角色权限成功，采用全量替换语义</t>
         </is>
       </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>存在目标角色与菜单权限</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>1. 提交新的 permissions 数组
 2. 再次查询角色权限</t>
         </is>
       </c>
-      <c r="J75" s="2" t="inlineStr">
+      <c r="J77" s="2" t="inlineStr">
         <is>
           <t>{"permissions":["admin:users:list","admin:users:create"]}</t>
         </is>
       </c>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr">
         <is>
           <t>返回“权限配置已保存”；再次查询结果与提交内容完全一致。</t>
         </is>
       </c>
-      <c r="L75" s="2" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>接口文档 §21 更新角色权限；接口差异提醒第 8 条；PRD §3.5.2</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>API-075</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/permissions</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G76" s="2" t="inlineStr">
+      <c r="G78" s="2" t="inlineStr">
         <is>
           <t>传空数组可清空角色所有权限</t>
         </is>
       </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H78" s="2" t="inlineStr">
         <is>
           <t>目标角色已有权限</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>1. 提交 permissions=[]
 2. 重新查询角色权限</t>
         </is>
       </c>
-      <c r="J76" s="2" t="inlineStr">
+      <c r="J78" s="2" t="inlineStr">
         <is>
           <t>{"permissions":[]}</t>
         </is>
       </c>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="K78" s="2" t="inlineStr">
         <is>
           <t>保存成功；角色权限被清空。</t>
         </is>
       </c>
-      <c r="L76" s="2" t="inlineStr">
+      <c r="L78" s="2" t="inlineStr">
         <is>
           <t>接口文档 §21 更新角色权限</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>API-076</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C79" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/roles/{id}/permissions</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G79" s="2" t="inlineStr">
         <is>
           <t>传入不存在权限标识时后端忽略而不报错</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H79" s="2" t="inlineStr">
         <is>
           <t>目标角色存在</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>1. 提交有效权限 + 无效权限组合
 2. 再次查询角色权限</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="J79" s="2" t="inlineStr">
         <is>
           <t>{"permissions":["admin:users:list","not:exists:permission"]}</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="K79" s="2" t="inlineStr">
         <is>
           <t>接口保存成功；无效权限不会被持久化，有效权限正常生效。</t>
         </is>
       </c>
-      <c r="L77" s="2" t="inlineStr">
+      <c r="L79" s="2" t="inlineStr">
         <is>
           <t>接口文档 §21 更新角色权限</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>API-077</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C80" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/tree</t>
         </is>
       </c>
-      <c r="D78" s="2" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G78" s="2" t="inlineStr">
+      <c r="G80" s="2" t="inlineStr">
         <is>
           <t>获取完整菜单树默认不包含停用节点</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H80" s="2" t="inlineStr">
         <is>
           <t>具备 admin:menus:list 权限</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
+      <c r="I80" s="2" t="inlineStr">
         <is>
           <t>1. 调用接口，不传 include_disabled
 2. 检查结果</t>
         </is>
       </c>
-      <c r="J78" s="2" t="inlineStr">
+      <c r="J80" s="2" t="inlineStr">
         <is>
           <t>include_disabled=false</t>
         </is>
       </c>
-      <c r="K78" s="2" t="inlineStr">
+      <c r="K80" s="2" t="inlineStr">
         <is>
           <t>返回完整菜单树，但默认不含停用节点；children 固定为数组。</t>
         </is>
       </c>
-      <c r="L78" s="2" t="inlineStr">
+      <c r="L80" s="2" t="inlineStr">
         <is>
           <t>接口文档 §22 获取完整菜单树</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>API-078</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/tree</t>
         </is>
       </c>
-      <c r="D79" s="2" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E81" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr">
+      <c r="G81" s="2" t="inlineStr">
         <is>
           <t>菜单管理页场景 include_disabled=true 可返回停用节点</t>
         </is>
       </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H81" s="2" t="inlineStr">
         <is>
           <t>存在停用菜单节点</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
+      <c r="I81" s="2" t="inlineStr">
         <is>
           <t>1. 传 include_disabled=true
 2. 检查返回</t>
         </is>
       </c>
-      <c r="J79" s="2" t="inlineStr">
+      <c r="J81" s="2" t="inlineStr">
         <is>
           <t>include_disabled=true</t>
         </is>
       </c>
-      <c r="K79" s="2" t="inlineStr">
+      <c r="K81" s="2" t="inlineStr">
         <is>
           <t>结果中包含停用节点，并带 status/status_label。</t>
         </is>
       </c>
-      <c r="L79" s="2" t="inlineStr">
+      <c r="L81" s="2" t="inlineStr">
         <is>
           <t>接口文档 §22 获取完整菜单树</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>API-079</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C82" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G82" s="2" t="inlineStr">
         <is>
           <t>新建根目录节点成功</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H82" s="2" t="inlineStr">
         <is>
           <t>具备 admin:menus:create 权限</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>1. parent_id 置空，新建目录节点
 2. 检查返回</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
+      <c r="J82" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":null,"type":1,"name":"帮助中心","permission":"help","sort":100,"status":1}</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr">
+      <c r="K82" s="2" t="inlineStr">
         <is>
           <t>目录节点创建成功。</t>
         </is>
       </c>
-      <c r="L80" s="2" t="inlineStr">
+      <c r="L82" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.2</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>API-080</t>
         </is>
       </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>新建菜单项节点时 route_path 和 component 必填</t>
         </is>
       </c>
-      <c r="H81" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>存在父目录</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
+      <c r="I83" s="2" t="inlineStr">
         <is>
           <t>1. 创建 type=2 菜单项
 2. 检查返回</t>
         </is>
       </c>
-      <c r="J81" s="2" t="inlineStr">
+      <c r="J83" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":1,"type":2,"name":"用户管理","permission":"admin:users:list","route_path":"/admin/users","component":"features/users/UserListPage","icon":"Users","sort":1,"status":1}</t>
         </is>
       </c>
-      <c r="K81" s="2" t="inlineStr">
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>菜单项创建成功；返回 id/name/permission/created_at。</t>
         </is>
       </c>
-      <c r="L81" s="2" t="inlineStr">
+      <c r="L83" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.2</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>API-081</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t>新建按钮节点成功</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>存在菜单项父节点</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>1. 以菜单项为父节点创建 type=3 按钮
 2. 检查返回</t>
         </is>
       </c>
-      <c r="J82" s="2" t="inlineStr">
+      <c r="J84" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":2,"type":3,"name":"新建用户","permission":"admin:users:create","sort":1,"status":1}</t>
         </is>
       </c>
-      <c r="K82" s="2" t="inlineStr">
+      <c r="K84" s="2" t="inlineStr">
         <is>
           <t>按钮节点创建成功。</t>
         </is>
       </c>
-      <c r="L82" s="2" t="inlineStr">
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.2</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>API-082</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t>权限标识重复时阻止保存</t>
         </is>
       </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>已存在相同 permission 节点</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>1. 使用重复 permission 创建节点
 2. 检查响应</t>
         </is>
       </c>
-      <c r="J83" s="2" t="inlineStr">
+      <c r="J85" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":1,"type":2,"name":"用户管理2","permission":"admin:users:list","route_path":"/admin/users2","component":"features/users/UserListPage","sort":2,"status":1}</t>
         </is>
       </c>
-      <c r="K83" s="2" t="inlineStr">
+      <c r="K85" s="2" t="inlineStr">
         <is>
           <t>返回 1001，message 为“权限标识已存在”。</t>
         </is>
       </c>
-      <c r="L83" s="2" t="inlineStr">
+      <c r="L85" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>API-083</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t>按钮节点不能直接挂在目录下</t>
         </is>
       </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>存在目录父节点</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
+      <c r="I86" s="2" t="inlineStr">
         <is>
           <t>1. parent_id 指向目录节点
 2. 创建 type=3 按钮</t>
         </is>
       </c>
-      <c r="J84" s="2" t="inlineStr">
+      <c r="J86" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":1,"type":3,"name":"非法按钮","permission":"admin:invalid:create","sort":1,"status":1}</t>
         </is>
       </c>
-      <c r="K84" s="2" t="inlineStr">
+      <c r="K86" s="2" t="inlineStr">
         <is>
           <t>返回 1001，message 为“按钮类型节点只能挂载在菜单项下”。</t>
         </is>
       </c>
-      <c r="L84" s="2" t="inlineStr">
+      <c r="L86" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>API-084</t>
         </is>
       </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t>菜单树最大仅支持 3 级</t>
         </is>
       </c>
-      <c r="H85" s="2" t="inlineStr">
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>已存在目录→菜单项→按钮 三级结构</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
+      <c r="I87" s="2" t="inlineStr">
         <is>
           <t>1. 以按钮为父节点继续创建子节点
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J85" s="2" t="inlineStr">
+      <c r="J87" s="2" t="inlineStr">
         <is>
           <t>{"parent_id":10,"type":3,"name":"四级按钮","permission":"admin:level4:create","sort":1,"status":1}</t>
         </is>
       </c>
-      <c r="K85" s="2" t="inlineStr">
+      <c r="K87" s="2" t="inlineStr">
         <is>
           <t>返回 1001，message 为“菜单树最多支持 3 级”。</t>
         </is>
       </c>
-      <c r="L85" s="2" t="inlineStr">
+      <c r="L87" s="2" t="inlineStr">
         <is>
           <t>接口文档 §23 新建菜单节点；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>API-085</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}</t>
         </is>
       </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G86" s="2" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t>编辑菜单节点成功</t>
         </is>
       </c>
-      <c r="H86" s="2" t="inlineStr">
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>存在目标菜单节点</t>
         </is>
       </c>
-      <c r="I86" s="2" t="inlineStr">
+      <c r="I88" s="2" t="inlineStr">
         <is>
           <t>1. 修改名称、路由、组件、排序、状态、备注
 2. 提交</t>
         </is>
       </c>
-      <c r="J86" s="2" t="inlineStr">
+      <c r="J88" s="2" t="inlineStr">
         <is>
           <t>{"name":"用户管理-新","route_path":"/admin/users","component":"features/users/UserListPage","icon":"Users","sort":10,"status":1,"remark":"说明"}</t>
         </is>
       </c>
-      <c r="K86" s="2" t="inlineStr">
+      <c r="K88" s="2" t="inlineStr">
         <is>
           <t>节点信息更新成功。</t>
         </is>
       </c>
-      <c r="L86" s="2" t="inlineStr">
+      <c r="L88" s="2" t="inlineStr">
         <is>
           <t>接口文档 §24 编辑菜单节点</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>API-086</t>
         </is>
       </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>PUT</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t>编辑菜单节点时 permission 和 type 传入也会被忽略</t>
         </is>
       </c>
-      <c r="H87" s="2" t="inlineStr">
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>存在目标节点</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr">
+      <c r="I89" s="2" t="inlineStr">
         <is>
           <t>1. 编辑时同时传 permission 与 type
 2. 查询详情或树</t>
         </is>
       </c>
-      <c r="J87" s="2" t="inlineStr">
+      <c r="J89" s="2" t="inlineStr">
         <is>
           <t>{"name":"用户管理","permission":"changed:permission","type":1,"route_path":"/admin/users","component":"features/users/UserListPage","sort":1,"status":1}</t>
         </is>
       </c>
-      <c r="K87" s="2" t="inlineStr">
+      <c r="K89" s="2" t="inlineStr">
         <is>
           <t>接口忽略 permission 与 type 修改；原值保持不变。</t>
         </is>
       </c>
-      <c r="L87" s="2" t="inlineStr">
+      <c r="L89" s="2" t="inlineStr">
         <is>
           <t>接口文档 §24 编辑菜单节点；接口差异提醒第 9 条</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>API-087</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}/status</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t>停用父节点时子节点同步停用并返回受影响节点数</t>
         </is>
       </c>
-      <c r="H88" s="2" t="inlineStr">
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>目标父节点下存在多级子节点</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr">
+      <c r="I90" s="2" t="inlineStr">
         <is>
           <t>1. 对父节点提交 status=2
 2. 查询菜单树</t>
         </is>
       </c>
-      <c r="J88" s="2" t="inlineStr">
+      <c r="J90" s="2" t="inlineStr">
         <is>
           <t>{"status":2}</t>
         </is>
       </c>
-      <c r="K88" s="2" t="inlineStr">
+      <c r="K90" s="2" t="inlineStr">
         <is>
           <t>返回 affected_count&gt;=父节点及全部子节点数量；父节点和子节点均为停用。</t>
         </is>
       </c>
-      <c r="L88" s="2" t="inlineStr">
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>接口文档 §25 切换菜单状态；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="2" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>API-088</t>
         </is>
       </c>
-      <c r="B89" s="2" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}/status</t>
         </is>
       </c>
-      <c r="D89" s="2" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>PATCH</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
+      <c r="E91" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G89" s="2" t="inlineStr">
+      <c r="G91" s="2" t="inlineStr">
         <is>
           <t>启用父节点时子节点状态不自动恢复</t>
         </is>
       </c>
-      <c r="H89" s="2" t="inlineStr">
+      <c r="H91" s="2" t="inlineStr">
         <is>
           <t>父节点及其子节点已全部停用</t>
         </is>
       </c>
-      <c r="I89" s="2" t="inlineStr">
+      <c r="I91" s="2" t="inlineStr">
         <is>
           <t>1. 先启用父节点
 2. 再查询树结构</t>
         </is>
       </c>
-      <c r="J89" s="2" t="inlineStr">
+      <c r="J91" s="2" t="inlineStr">
         <is>
           <t>{"status":1}</t>
         </is>
       </c>
-      <c r="K89" s="2" t="inlineStr">
+      <c r="K91" s="2" t="inlineStr">
         <is>
           <t>父节点恢复启用；原被连带停用的子节点仍保持停用，需要手动启用。</t>
         </is>
       </c>
-      <c r="L89" s="2" t="inlineStr">
+      <c r="L91" s="2" t="inlineStr">
         <is>
           <t>接口文档 §25 切换菜单状态；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>API-089</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G92" s="2" t="inlineStr">
         <is>
           <t>删除未被引用且无子节点的菜单成功</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr">
+      <c r="H92" s="2" t="inlineStr">
         <is>
           <t>目标节点无子节点且未被角色引用</t>
         </is>
       </c>
-      <c r="I90" s="2" t="inlineStr">
+      <c r="I92" s="2" t="inlineStr">
         <is>
           <t>1. 调用删除接口
 2. 检查树中节点消失</t>
         </is>
       </c>
-      <c r="J90" s="2" t="inlineStr">
+      <c r="J92" s="2" t="inlineStr">
         <is>
           <t>id=deletable_menu_id</t>
         </is>
       </c>
-      <c r="K90" s="2" t="inlineStr">
+      <c r="K92" s="2" t="inlineStr">
         <is>
           <t>返回“菜单已删除”；data=null。</t>
         </is>
       </c>
-      <c r="L90" s="2" t="inlineStr">
+      <c r="L92" s="2" t="inlineStr">
         <is>
           <t>接口文档 §26 删除菜单节点</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>API-090</t>
         </is>
       </c>
-      <c r="B91" s="2" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C91" s="2" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G91" s="2" t="inlineStr">
+      <c r="G93" s="2" t="inlineStr">
         <is>
           <t>被角色引用的菜单节点不可删除</t>
         </is>
       </c>
-      <c r="H91" s="2" t="inlineStr">
+      <c r="H93" s="2" t="inlineStr">
         <is>
           <t>目标节点已绑定到角色权限</t>
         </is>
       </c>
-      <c r="I91" s="2" t="inlineStr">
+      <c r="I93" s="2" t="inlineStr">
         <is>
           <t>1. 删除被角色引用的节点
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J91" s="2" t="inlineStr">
+      <c r="J93" s="2" t="inlineStr">
         <is>
           <t>id=referenced_menu_id</t>
         </is>
       </c>
-      <c r="K91" s="2" t="inlineStr">
+      <c r="K93" s="2" t="inlineStr">
         <is>
           <t>返回 1005，message 为“该菜单已被 N 个角色引用，请先解绑后再删除”。</t>
         </is>
       </c>
-      <c r="L91" s="2" t="inlineStr">
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>接口文档 §26 删除菜单节点；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>API-091</t>
         </is>
       </c>
-      <c r="B92" s="2" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>菜单与权限</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/menus/{id}</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="F94" s="2" t="inlineStr">
         <is>
           <t>业务规则</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr">
+      <c r="G94" s="2" t="inlineStr">
         <is>
           <t>存在子节点的父节点不可直接删除</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr">
+      <c r="H94" s="2" t="inlineStr">
         <is>
           <t>目标节点存在子节点</t>
         </is>
       </c>
-      <c r="I92" s="2" t="inlineStr">
+      <c r="I94" s="2" t="inlineStr">
         <is>
           <t>1. 删除父节点
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J92" s="2" t="inlineStr">
+      <c r="J94" s="2" t="inlineStr">
         <is>
           <t>id=parent_menu_id</t>
         </is>
       </c>
-      <c r="K92" s="2" t="inlineStr">
+      <c r="K94" s="2" t="inlineStr">
         <is>
           <t>返回 1005，message 为“请先删除子节点后再删除父节点”。</t>
         </is>
       </c>
-      <c r="L92" s="2" t="inlineStr">
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>接口文档 §26 删除菜单节点；PRD §3.4.4</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>API-092</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F95" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="G95" s="2" t="inlineStr">
         <is>
           <t>审计日志列表分页查询成功</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
+      <c r="H95" s="2" t="inlineStr">
         <is>
           <t>具备 admin:audit-logs:list 权限</t>
         </is>
       </c>
-      <c r="I93" s="2" t="inlineStr">
+      <c r="I95" s="2" t="inlineStr">
         <is>
           <t>1. 调用审计日志列表
 2. 检查分页与字段</t>
         </is>
       </c>
-      <c r="J93" s="2" t="inlineStr">
+      <c r="J95" s="2" t="inlineStr">
         <is>
           <t>page=1&amp;per_page=20</t>
         </is>
       </c>
-      <c r="K93" s="2" t="inlineStr">
+      <c r="K95" s="2" t="inlineStr">
         <is>
           <t>返回日志列表，含 log_type、operator、action、object、result、created_at 等字段。</t>
         </is>
       </c>
-      <c r="L93" s="2" t="inlineStr">
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>接口文档 §27 审计日志列表；PRD §3.6.2</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>API-093</t>
         </is>
       </c>
-      <c r="B94" s="2" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C94" s="2" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs</t>
         </is>
       </c>
-      <c r="D94" s="2" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>筛选</t>
         </is>
       </c>
-      <c r="G94" s="2" t="inlineStr">
+      <c r="G96" s="2" t="inlineStr">
         <is>
           <t>支持按日志类型、操作人、对象类型、时间范围筛选</t>
         </is>
       </c>
-      <c r="H94" s="2" t="inlineStr">
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>存在多类日志数据</t>
         </is>
       </c>
-      <c r="I94" s="2" t="inlineStr">
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>1. 组合传入筛选条件
 2. 校验结果集</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr">
+      <c r="J96" s="2" t="inlineStr">
         <is>
           <t>log_type=user_permission&amp;operator_id=1&amp;object_type=user&amp;start_time=2026-03-01T00:00:00Z&amp;end_time=2026-03-31T23:59:59Z</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr">
+      <c r="K96" s="2" t="inlineStr">
         <is>
           <t>返回结果同时满足筛选条件。</t>
         </is>
       </c>
-      <c r="L94" s="2" t="inlineStr">
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>接口文档 §27 审计日志列表；PRD §3.6.2</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>API-094</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr">
+      <c r="E97" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>校验</t>
         </is>
       </c>
-      <c r="G95" s="2" t="inlineStr">
+      <c r="G97" s="2" t="inlineStr">
         <is>
           <t>时间筛选格式非法时返回参数错误</t>
         </is>
       </c>
-      <c r="H95" s="2" t="inlineStr">
+      <c r="H97" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="I95" s="2" t="inlineStr">
+      <c r="I97" s="2" t="inlineStr">
         <is>
           <t>1. 传非法 start_time/end_time
 2. 查看响应</t>
         </is>
       </c>
-      <c r="J95" s="2" t="inlineStr">
+      <c r="J97" s="2" t="inlineStr">
         <is>
           <t>start_time=2026/03/01 00:00:00</t>
         </is>
       </c>
-      <c r="K95" s="2" t="inlineStr">
+      <c r="K97" s="2" t="inlineStr">
         <is>
           <t>返回 1001，提示时间格式需为 UTC ISO 8601。</t>
         </is>
       </c>
-      <c r="L95" s="2" t="inlineStr">
+      <c r="L97" s="2" t="inlineStr">
         <is>
           <t>接口文档 §27 审计日志列表；接口文档-时间格式</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>API-095</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs/{id}</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>正向</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr">
         <is>
           <t>审计日志详情可返回字段级 before/after 变更值</t>
         </is>
       </c>
-      <c r="H96" s="2" t="inlineStr">
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>存在编辑类日志</t>
         </is>
       </c>
-      <c r="I96" s="2" t="inlineStr">
+      <c r="I98" s="2" t="inlineStr">
         <is>
           <t>1. 调用日志详情接口
 2. 检查 before_value/after_value</t>
         </is>
       </c>
-      <c r="J96" s="2" t="inlineStr">
+      <c r="J98" s="2" t="inlineStr">
         <is>
           <t>id=1001</t>
         </is>
       </c>
-      <c r="K96" s="2" t="inlineStr">
+      <c r="K98" s="2" t="inlineStr">
         <is>
           <t>返回变更前后 JSON、source_page、request_id、result 等字段。</t>
         </is>
       </c>
-      <c r="L96" s="2" t="inlineStr">
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>接口文档 §28 审计日志详情；PRD §3.6.3</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
         <is>
           <t>API-096</t>
         </is>
       </c>
-      <c r="B97" s="2" t="inlineStr">
+      <c r="B99" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C97" s="2" t="inlineStr">
+      <c r="C99" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs/{id}</t>
         </is>
       </c>
-      <c r="D97" s="2" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>边界</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr">
+      <c r="G99" s="2" t="inlineStr">
         <is>
           <t>新建/删除类日志支持 before_value 或 after_value 为 null</t>
         </is>
       </c>
-      <c r="H97" s="2" t="inlineStr">
+      <c r="H99" s="2" t="inlineStr">
         <is>
           <t>存在 create 或 delete 类型日志</t>
         </is>
       </c>
-      <c r="I97" s="2" t="inlineStr">
+      <c r="I99" s="2" t="inlineStr">
         <is>
           <t>1. 查询新建日志详情
 2. 查询删除日志详情</t>
         </is>
       </c>
-      <c r="J97" s="2" t="inlineStr">
+      <c r="J99" s="2" t="inlineStr">
         <is>
           <t>id=create_log_id / delete_log_id</t>
         </is>
       </c>
-      <c r="K97" s="2" t="inlineStr">
+      <c r="K99" s="2" t="inlineStr">
         <is>
           <t>新建日志 before_value=null；删除日志 after_value=null；失败原因无值时 fail_reason=null。</t>
         </is>
       </c>
-      <c r="L97" s="2" t="inlineStr">
+      <c r="L99" s="2" t="inlineStr">
         <is>
           <t>接口文档 §28 审计日志详情</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
         <is>
           <t>API-097</t>
         </is>
       </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>审计日志</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>/api/v1/admin/audit-logs/{id}</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>异常</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G100" s="2" t="inlineStr">
         <is>
           <t>不存在日志详情返回 1004</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
+      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="I100" s="2" t="inlineStr">
         <is>
           <t>1. 查询不存在日志 id
 2. 检查响应</t>
         </is>
       </c>
-      <c r="J98" s="2" t="inlineStr">
+      <c r="J100" s="2" t="inlineStr">
         <is>
           <t>id=999999</t>
         </is>
       </c>
-      <c r="K98" s="2" t="inlineStr">
+      <c r="K100" s="2" t="inlineStr">
         <is>
           <t>返回 1004。</t>
         </is>
       </c>
-      <c r="L98" s="2" t="inlineStr">
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>接口文档-公共错误码；接口文档 §28 审计日志详情</t>
         </is>
@@ -6809,7 +6935,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">

</xml_diff>